<commit_message>
Made milestones from lecture 8 in NSC and updated a lot in project
</commit_message>
<xml_diff>
--- a/Projekt/Lydfiler/impulseResponseMeasurerData/omniPower/excelOfValues.xlsx
+++ b/Projekt/Lydfiler/impulseResponseMeasurerData/omniPower/excelOfValues.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Christian Lykke\Documents\Skole\Aalborg Universitet\CEAIVS8\Projekt\Lydfiler\impulseResponseMeasurerData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Christian Lykke\Documents\Skole\Aalborg Universitet\CEAIVS8\Projekt\Lydfiler\impulseResponseMeasurerData\omniPower\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA05F9A5-994E-4398-890C-761546F5A522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A7CE28B-6C2F-42C9-AA63-4137CA938838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21240" xr2:uid="{4D278BF0-5144-496E-BFC7-CFB5FE610154}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="20">
   <si>
     <t>Frequency</t>
   </si>
@@ -90,6 +90,12 @@
   </si>
   <si>
     <t>MLS</t>
+  </si>
+  <si>
+    <t>Comparison</t>
+  </si>
+  <si>
+    <t>undocumented</t>
   </si>
 </sst>
 </file>
@@ -483,21 +489,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3EE57F2-BDDA-4B86-B811-3E649D61B89B}">
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:Y32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
       <c r="L1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -558,8 +567,11 @@
       <c r="U2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -621,11 +633,14 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="L4" s="2"/>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="W4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>50</v>
       </c>
@@ -686,8 +701,14 @@
       <c r="U5">
         <v>0.19364999999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="W5">
+        <v>0.96</v>
+      </c>
+      <c r="Y5">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>63</v>
       </c>
@@ -748,8 +769,11 @@
       <c r="U6">
         <v>0.37319999999999998</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y6">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>80</v>
       </c>
@@ -810,8 +834,11 @@
       <c r="U7">
         <v>0.47742000000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y7">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>100</v>
       </c>
@@ -872,8 +899,11 @@
       <c r="U8">
         <v>0.53544999999999998</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y8">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>125</v>
       </c>
@@ -934,8 +964,11 @@
       <c r="U9">
         <v>0.70289000000000001</v>
       </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y9">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>160</v>
       </c>
@@ -996,8 +1029,12 @@
       <c r="U10">
         <v>0.76812000000000002</v>
       </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y10">
+        <f>(F10+Q10)/2</f>
+        <v>0.75429000000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>200</v>
       </c>
@@ -1058,8 +1095,12 @@
       <c r="U11">
         <v>0.74341999999999997</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y11">
+        <f>(F11+Q11)/2</f>
+        <v>0.64614499999999997</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>250</v>
       </c>
@@ -1120,8 +1161,12 @@
       <c r="U12">
         <v>0.83843000000000001</v>
       </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y12">
+        <f>(F12+Q12)/2</f>
+        <v>0.59955500000000006</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>315</v>
       </c>
@@ -1182,8 +1227,12 @@
       <c r="U13">
         <v>0.84138000000000002</v>
       </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y13">
+        <f>(F13+Q13)/2</f>
+        <v>0.56536500000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>400</v>
       </c>
@@ -1244,8 +1293,12 @@
       <c r="U14">
         <v>0.88056999999999996</v>
       </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y14">
+        <f>(F14+Q14)/2</f>
+        <v>0.559805</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>500</v>
       </c>
@@ -1306,8 +1359,12 @@
       <c r="U15">
         <v>0.85575999999999997</v>
       </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y15">
+        <f>(F15+Q15)/2</f>
+        <v>0.6475200000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>630</v>
       </c>
@@ -1368,8 +1425,12 @@
       <c r="U16">
         <v>0.82547000000000004</v>
       </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y16">
+        <f>(F16+Q16)/2</f>
+        <v>0.6769750000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>800</v>
       </c>
@@ -1430,8 +1491,12 @@
       <c r="U17">
         <v>0.82198000000000004</v>
       </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y17">
+        <f>(F17+Q17)/2</f>
+        <v>0.69895499999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>1000</v>
       </c>
@@ -1492,8 +1557,12 @@
       <c r="U18">
         <v>0.81794</v>
       </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y18">
+        <f>(F18+Q18)/2</f>
+        <v>0.70206999999999997</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>1250</v>
       </c>
@@ -1554,8 +1623,12 @@
       <c r="U19">
         <v>0.81545999999999996</v>
       </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y19">
+        <f>(F19+Q19)/2</f>
+        <v>0.72611999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>1600</v>
       </c>
@@ -1616,8 +1689,12 @@
       <c r="U20">
         <v>0.81045999999999996</v>
       </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y20">
+        <f>(F20+Q20)/2</f>
+        <v>0.73229</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>2000</v>
       </c>
@@ -1678,8 +1755,12 @@
       <c r="U21">
         <v>0.80052000000000001</v>
       </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y21">
+        <f>(F21+Q21)/2</f>
+        <v>0.75208000000000008</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>2500</v>
       </c>
@@ -1740,8 +1821,12 @@
       <c r="U22">
         <v>0.79468000000000005</v>
       </c>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y22">
+        <f>(F22+Q22)/2</f>
+        <v>0.76478500000000005</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>3150</v>
       </c>
@@ -1802,8 +1887,12 @@
       <c r="U23">
         <v>0.78952</v>
       </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y23">
+        <f>(F23+Q23)/2</f>
+        <v>0.78190000000000004</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>4000</v>
       </c>
@@ -1864,8 +1953,12 @@
       <c r="U24">
         <v>0.79991999999999996</v>
       </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y24">
+        <f>(F24+Q24)/2</f>
+        <v>0.75202999999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>5000</v>
       </c>
@@ -1926,8 +2019,12 @@
       <c r="U25">
         <v>0.81840000000000002</v>
       </c>
-    </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y25">
+        <f>(F25+Q25)/2</f>
+        <v>0.70745999999999998</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>6300</v>
       </c>
@@ -1988,8 +2085,12 @@
       <c r="U26">
         <v>0.83704999999999996</v>
       </c>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y26">
+        <f>(F26+Q26)/2</f>
+        <v>0.65663000000000005</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>8000</v>
       </c>
@@ -2050,8 +2151,12 @@
       <c r="U27">
         <v>0.88907999999999998</v>
       </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y27">
+        <f>(F27+Q27)/2</f>
+        <v>0.55407499999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>10000</v>
       </c>
@@ -2112,8 +2217,12 @@
       <c r="U28">
         <v>0.92278000000000004</v>
       </c>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y28">
+        <f>(F28+Q28)/2</f>
+        <v>0.47575999999999996</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>12500</v>
       </c>
@@ -2174,8 +2283,12 @@
       <c r="U29">
         <v>0.94486000000000003</v>
       </c>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y29">
+        <f>(F29+Q29)/2</f>
+        <v>0.40989500000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>16000</v>
       </c>
@@ -2236,8 +2349,11 @@
       <c r="U30">
         <v>0.94881000000000004</v>
       </c>
-    </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y30">
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>20000</v>
       </c>
@@ -2298,8 +2414,11 @@
       <c r="U31">
         <v>0.92083999999999999</v>
       </c>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="Y31">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>16</v>
       </c>
@@ -2332,7 +2451,7 @@
         <v>7.2232117647058836</v>
       </c>
       <c r="I32">
-        <f t="shared" ref="C32:J32" si="0">SUM(I12:I28)/17</f>
+        <f t="shared" ref="I32:J32" si="0">SUM(I12:I28)/17</f>
         <v>0.67677235294117655</v>
       </c>
       <c r="J32">
@@ -2377,6 +2496,10 @@
       <c r="U32">
         <f t="shared" si="1"/>
         <v>0.83290588235294105</v>
+      </c>
+      <c r="Y32">
+        <f>(F32+Q32)/2</f>
+        <v>0.65139532142857159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>